<commit_message>
etsy: assinaturas sem cara de IA (ingles e frances, status em palavras, fotos novas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/subscriptions/Abonnements-Suivi.xlsx
+++ b/etsy/subscriptions/Abonnements-Suivi.xlsx
@@ -106,7 +106,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -115,8 +115,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F4EF"/>
-        <bgColor rgb="00F6F4EF"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,12 +129,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF4C2"/>
         <bgColor rgb="00FFF4C2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -172,16 +166,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </bottom>
     </border>
   </borders>
@@ -193,15 +187,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="10" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -211,20 +205,22 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -233,7 +229,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -241,6 +237,14 @@
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D8F0DC"/>
+          <bgColor rgb="00D8F0DC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -267,14 +271,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="00FFE2B8"/>
           <bgColor rgb="00FFE2B8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00D8F0DC"/>
-          <bgColor rgb="00D8F0DC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -668,7 +664,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Où part l’argent chaque mois</t>
+          <t>Ce que coûtent vos abonnements</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -785,7 +781,7 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>par an pour des choses que vous n’utilisez pas</t>
+          <t>par an pour des choses que vous n'utilisez pas</t>
         </is>
       </c>
       <c r="G8" s="1" t="n"/>
@@ -863,7 +859,7 @@
       </c>
       <c r="G11" s="1" t="n"/>
       <c r="H11" s="19">
-        <f>COUNTIFS(Abonnements!$L$6:$L$55,"⚠*")&amp;" essai(s) gratuit(s) bientôt payant(s)"</f>
+        <f>IF(COUNTIFS(Abonnements!$L$6:$L$55,"Fin de*")=0,"Aucun essai gratuit ne va devenir payant",IF(COUNTIFS(Abonnements!$L$6:$L$55,"Fin de*")=1,"1 essai gratuit va bientôt devenir payant",COUNTIFS(Abonnements!$L$6:$L$55,"Fin de*")&amp;" essais gratuits vont bientôt devenir payants"))</f>
         <v/>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -920,7 +916,7 @@
       </c>
       <c r="G13" s="1" t="n"/>
       <c r="H13" s="20">
-        <f>COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 0 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 1 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 2 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 3 jour*")&amp;" renouvellement(s) dans les 3 jours"</f>
+        <f>IF((COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 0 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 1 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 2 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 3 jour*"))=0,"Aucun renouvellement dans les 3 jours",IF((COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 0 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 1 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 2 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 3 jour*"))=1,"1 renouvellement",(COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 0 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 1 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 2 jour*")+COUNTIFS(Abonnements!$L$6:$L$55,"Renouvellement dans 3 jour*"))&amp;" renouvellements")&amp;" dans les 3 jours")</f>
         <v/>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -977,7 +973,7 @@
       </c>
       <c r="G15" s="1" t="n"/>
       <c r="H15" s="20">
-        <f>COUNTIFS(Abonnements!$L$6:$L$55,"💤*")&amp;" abonnement(s) pas utilisé(s) depuis un mois"</f>
+        <f>IF(COUNTIFS(Abonnements!$L$6:$L$55,"Pas utilisé*")=0,"Tout a servi le mois dernier",IF(COUNTIFS(Abonnements!$L$6:$L$55,"Pas utilisé*")=1,"1 abonnement n'a pas servi",COUNTIFS(Abonnements!$L$6:$L$55,"Pas utilisé*")&amp;" abonnements n'ont pas servi")&amp;" depuis plus d'un mois")</f>
         <v/>
       </c>
       <c r="I15" s="1" t="n"/>
@@ -1034,7 +1030,7 @@
       </c>
       <c r="G17" s="1" t="n"/>
       <c r="H17" s="21">
-        <f>COUNTIFS(Abonnements!$I$6:$I$55,"Décider")&amp;" encore à décider : garder ou annuler ?"</f>
+        <f>IF(COUNTIFS(Abonnements!$I$6:$I$55,"Décider")=0,"Plus rien à décider",IF(COUNTIFS(Abonnements!$I$6:$I$55,"Décider")=1,"1 abonnement",COUNTIFS(Abonnements!$I$6:$I$55,"Décider")&amp;" abonnements")&amp;" encore à décider : garder ou annuler")</f>
         <v/>
       </c>
       <c r="I17" s="1" t="n"/>
@@ -1754,6 +1750,26 @@
       <c r="I79" s="1" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H11">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>LEFT(H11,5)="Aucun"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H13">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>LEFT(H13,5)="Aucun"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H15">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>LEFT(H15,4)="Tout"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>LEFT(H17,4)="Plus"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1801,7 +1817,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Tous vos abonnements, au même endroit</t>
+          <t>Vos abonnements</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -1932,8 +1948,10 @@
       <c r="F6" s="25" t="n">
         <v>46265</v>
       </c>
-      <c r="G6" s="24" t="b">
-        <v>0</v>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H6" s="25" t="n">
         <v>46292</v>
@@ -1952,7 +1970,7 @@
         <v/>
       </c>
       <c r="L6" s="26">
-        <f>IF(OR(B6="",F6=""),"",IF(I6="Annuler","✗ À annuler sous "&amp;(IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G6=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H6&lt;&gt;"",TODAY()-H6&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H6)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B6="",F6=""),"",IF(I6="Annuler","À annuler sous "&amp;(IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G6="Oui","Fin de l'essai dans "&amp;(IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H6&lt;&gt;"",TODAY()-H6&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H6)&amp;" jours","Renouvellement dans "&amp;(IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F6&gt;=TODAY(),F6,IF(E6="Hebdo",F6+7*ROUNDUP((TODAY()-F6)/7,0),EDATE(F6,IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12))*ROUNDUP((DATEDIF(F6,TODAY(),"m")+1)/IF(E6="Mensuel",1,IF(E6="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M6" s="1" t="n"/>
@@ -1980,8 +1998,10 @@
       <c r="F7" s="25" t="n">
         <v>46281</v>
       </c>
-      <c r="G7" s="24" t="b">
-        <v>0</v>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H7" s="25" t="n">
         <v>46252</v>
@@ -2000,7 +2020,7 @@
         <v/>
       </c>
       <c r="L7" s="26">
-        <f>IF(OR(B7="",F7=""),"",IF(I7="Annuler","✗ À annuler sous "&amp;(IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G7=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H7&lt;&gt;"",TODAY()-H7&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H7)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B7="",F7=""),"",IF(I7="Annuler","À annuler sous "&amp;(IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G7="Oui","Fin de l'essai dans "&amp;(IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H7&lt;&gt;"",TODAY()-H7&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H7)&amp;" jours","Renouvellement dans "&amp;(IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F7&gt;=TODAY(),F7,IF(E7="Hebdo",F7+7*ROUNDUP((TODAY()-F7)/7,0),EDATE(F7,IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12))*ROUNDUP((DATEDIF(F7,TODAY(),"m")+1)/IF(E7="Mensuel",1,IF(E7="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M7" s="1" t="n"/>
@@ -2028,8 +2048,10 @@
       <c r="F8" s="25" t="n">
         <v>46290</v>
       </c>
-      <c r="G8" s="24" t="b">
-        <v>0</v>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H8" s="25" t="n">
         <v>46293</v>
@@ -2048,7 +2070,7 @@
         <v/>
       </c>
       <c r="L8" s="26">
-        <f>IF(OR(B8="",F8=""),"",IF(I8="Annuler","✗ À annuler sous "&amp;(IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G8=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H8&lt;&gt;"",TODAY()-H8&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H8)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B8="",F8=""),"",IF(I8="Annuler","À annuler sous "&amp;(IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G8="Oui","Fin de l'essai dans "&amp;(IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H8&lt;&gt;"",TODAY()-H8&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H8)&amp;" jours","Renouvellement dans "&amp;(IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F8&gt;=TODAY(),F8,IF(E8="Hebdo",F8+7*ROUNDUP((TODAY()-F8)/7,0),EDATE(F8,IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12))*ROUNDUP((DATEDIF(F8,TODAY(),"m")+1)/IF(E8="Mensuel",1,IF(E8="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M8" s="1" t="n"/>
@@ -2076,8 +2098,10 @@
       <c r="F9" s="25" t="n">
         <v>45933</v>
       </c>
-      <c r="G9" s="24" t="b">
-        <v>0</v>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H9" s="25" t="n">
         <v>46291</v>
@@ -2096,7 +2120,7 @@
         <v/>
       </c>
       <c r="L9" s="26">
-        <f>IF(OR(B9="",F9=""),"",IF(I9="Annuler","✗ À annuler sous "&amp;(IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G9=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H9&lt;&gt;"",TODAY()-H9&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H9)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B9="",F9=""),"",IF(I9="Annuler","À annuler sous "&amp;(IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G9="Oui","Fin de l'essai dans "&amp;(IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H9&lt;&gt;"",TODAY()-H9&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H9)&amp;" jours","Renouvellement dans "&amp;(IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F9&gt;=TODAY(),F9,IF(E9="Hebdo",F9+7*ROUNDUP((TODAY()-F9)/7,0),EDATE(F9,IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12))*ROUNDUP((DATEDIF(F9,TODAY(),"m")+1)/IF(E9="Mensuel",1,IF(E9="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M9" s="1" t="n"/>
@@ -2124,8 +2148,10 @@
       <c r="F10" s="25" t="n">
         <v>46273</v>
       </c>
-      <c r="G10" s="24" t="b">
-        <v>0</v>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H10" s="25" t="n">
         <v>46230</v>
@@ -2144,7 +2170,7 @@
         <v/>
       </c>
       <c r="L10" s="26">
-        <f>IF(OR(B10="",F10=""),"",IF(I10="Annuler","✗ À annuler sous "&amp;(IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G10=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H10&lt;&gt;"",TODAY()-H10&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H10)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B10="",F10=""),"",IF(I10="Annuler","À annuler sous "&amp;(IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G10="Oui","Fin de l'essai dans "&amp;(IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H10&lt;&gt;"",TODAY()-H10&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H10)&amp;" jours","Renouvellement dans "&amp;(IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F10&gt;=TODAY(),F10,IF(E10="Hebdo",F10+7*ROUNDUP((TODAY()-F10)/7,0),EDATE(F10,IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12))*ROUNDUP((DATEDIF(F10,TODAY(),"m")+1)/IF(E10="Mensuel",1,IF(E10="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M10" s="1" t="n"/>
@@ -2172,8 +2198,10 @@
       <c r="F11" s="25" t="n">
         <v>46288</v>
       </c>
-      <c r="G11" s="24" t="b">
-        <v>1</v>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
       </c>
       <c r="H11" s="25" t="n">
         <v>46288</v>
@@ -2192,7 +2220,7 @@
         <v/>
       </c>
       <c r="L11" s="26">
-        <f>IF(OR(B11="",F11=""),"",IF(I11="Annuler","✗ À annuler sous "&amp;(IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G11=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H11&lt;&gt;"",TODAY()-H11&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H11)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B11="",F11=""),"",IF(I11="Annuler","À annuler sous "&amp;(IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G11="Oui","Fin de l'essai dans "&amp;(IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H11&lt;&gt;"",TODAY()-H11&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H11)&amp;" jours","Renouvellement dans "&amp;(IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F11&gt;=TODAY(),F11,IF(E11="Hebdo",F11+7*ROUNDUP((TODAY()-F11)/7,0),EDATE(F11,IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12))*ROUNDUP((DATEDIF(F11,TODAY(),"m")+1)/IF(E11="Mensuel",1,IF(E11="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M11" s="1" t="n"/>
@@ -2220,8 +2248,10 @@
       <c r="F12" s="25" t="n">
         <v>46265</v>
       </c>
-      <c r="G12" s="24" t="b">
-        <v>1</v>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
       </c>
       <c r="H12" s="25" t="n">
         <v>46283</v>
@@ -2240,7 +2270,7 @@
         <v/>
       </c>
       <c r="L12" s="26">
-        <f>IF(OR(B12="",F12=""),"",IF(I12="Annuler","✗ À annuler sous "&amp;(IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G12=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H12&lt;&gt;"",TODAY()-H12&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H12)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B12="",F12=""),"",IF(I12="Annuler","À annuler sous "&amp;(IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G12="Oui","Fin de l'essai dans "&amp;(IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H12&lt;&gt;"",TODAY()-H12&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H12)&amp;" jours","Renouvellement dans "&amp;(IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F12&gt;=TODAY(),F12,IF(E12="Hebdo",F12+7*ROUNDUP((TODAY()-F12)/7,0),EDATE(F12,IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12))*ROUNDUP((DATEDIF(F12,TODAY(),"m")+1)/IF(E12="Mensuel",1,IF(E12="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M12" s="1" t="n"/>
@@ -2268,8 +2298,10 @@
       <c r="F13" s="25" t="n">
         <v>46284</v>
       </c>
-      <c r="G13" s="24" t="b">
-        <v>0</v>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H13" s="25" t="n">
         <v>46274</v>
@@ -2288,7 +2320,7 @@
         <v/>
       </c>
       <c r="L13" s="26">
-        <f>IF(OR(B13="",F13=""),"",IF(I13="Annuler","✗ À annuler sous "&amp;(IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G13=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H13&lt;&gt;"",TODAY()-H13&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H13)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B13="",F13=""),"",IF(I13="Annuler","À annuler sous "&amp;(IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G13="Oui","Fin de l'essai dans "&amp;(IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H13&lt;&gt;"",TODAY()-H13&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H13)&amp;" jours","Renouvellement dans "&amp;(IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F13&gt;=TODAY(),F13,IF(E13="Hebdo",F13+7*ROUNDUP((TODAY()-F13)/7,0),EDATE(F13,IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12))*ROUNDUP((DATEDIF(F13,TODAY(),"m")+1)/IF(E13="Mensuel",1,IF(E13="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M13" s="1" t="n"/>
@@ -2297,7 +2329,7 @@
       <c r="A14" s="1" t="n"/>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>Site d’info</t>
+          <t>Site d'info</t>
         </is>
       </c>
       <c r="C14" s="22" t="inlineStr">
@@ -2316,8 +2348,10 @@
       <c r="F14" s="25" t="n">
         <v>46213</v>
       </c>
-      <c r="G14" s="24" t="b">
-        <v>0</v>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H14" s="25" t="n">
         <v>46260</v>
@@ -2336,7 +2370,7 @@
         <v/>
       </c>
       <c r="L14" s="26">
-        <f>IF(OR(B14="",F14=""),"",IF(I14="Annuler","✗ À annuler sous "&amp;(IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G14=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H14&lt;&gt;"",TODAY()-H14&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H14)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B14="",F14=""),"",IF(I14="Annuler","À annuler sous "&amp;(IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G14="Oui","Fin de l'essai dans "&amp;(IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H14&lt;&gt;"",TODAY()-H14&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H14)&amp;" jours","Renouvellement dans "&amp;(IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F14&gt;=TODAY(),F14,IF(E14="Hebdo",F14+7*ROUNDUP((TODAY()-F14)/7,0),EDATE(F14,IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12))*ROUNDUP((DATEDIF(F14,TODAY(),"m")+1)/IF(E14="Mensuel",1,IF(E14="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M14" s="1" t="n"/>
@@ -2364,8 +2398,10 @@
       <c r="F15" s="25" t="n">
         <v>46278</v>
       </c>
-      <c r="G15" s="24" t="b">
-        <v>0</v>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
       </c>
       <c r="H15" s="25" t="n">
         <v>46289</v>
@@ -2384,7 +2420,7 @@
         <v/>
       </c>
       <c r="L15" s="26">
-        <f>IF(OR(B15="",F15=""),"",IF(I15="Annuler","✗ À annuler sous "&amp;(IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G15=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H15&lt;&gt;"",TODAY()-H15&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H15)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B15="",F15=""),"",IF(I15="Annuler","À annuler sous "&amp;(IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G15="Oui","Fin de l'essai dans "&amp;(IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H15&lt;&gt;"",TODAY()-H15&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H15)&amp;" jours","Renouvellement dans "&amp;(IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F15&gt;=TODAY(),F15,IF(E15="Hebdo",F15+7*ROUNDUP((TODAY()-F15)/7,0),EDATE(F15,IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12))*ROUNDUP((DATEDIF(F15,TODAY(),"m")+1)/IF(E15="Mensuel",1,IF(E15="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M15" s="1" t="n"/>
@@ -2408,7 +2444,7 @@
         <v/>
       </c>
       <c r="L16" s="26">
-        <f>IF(OR(B16="",F16=""),"",IF(I16="Annuler","✗ À annuler sous "&amp;(IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G16=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H16&lt;&gt;"",TODAY()-H16&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H16)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B16="",F16=""),"",IF(I16="Annuler","À annuler sous "&amp;(IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G16="Oui","Fin de l'essai dans "&amp;(IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H16&lt;&gt;"",TODAY()-H16&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H16)&amp;" jours","Renouvellement dans "&amp;(IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F16&gt;=TODAY(),F16,IF(E16="Hebdo",F16+7*ROUNDUP((TODAY()-F16)/7,0),EDATE(F16,IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12))*ROUNDUP((DATEDIF(F16,TODAY(),"m")+1)/IF(E16="Mensuel",1,IF(E16="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M16" s="1" t="n"/>
@@ -2432,7 +2468,7 @@
         <v/>
       </c>
       <c r="L17" s="26">
-        <f>IF(OR(B17="",F17=""),"",IF(I17="Annuler","✗ À annuler sous "&amp;(IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G17=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H17&lt;&gt;"",TODAY()-H17&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H17)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B17="",F17=""),"",IF(I17="Annuler","À annuler sous "&amp;(IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G17="Oui","Fin de l'essai dans "&amp;(IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H17&lt;&gt;"",TODAY()-H17&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H17)&amp;" jours","Renouvellement dans "&amp;(IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F17&gt;=TODAY(),F17,IF(E17="Hebdo",F17+7*ROUNDUP((TODAY()-F17)/7,0),EDATE(F17,IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12))*ROUNDUP((DATEDIF(F17,TODAY(),"m")+1)/IF(E17="Mensuel",1,IF(E17="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M17" s="1" t="n"/>
@@ -2456,7 +2492,7 @@
         <v/>
       </c>
       <c r="L18" s="26">
-        <f>IF(OR(B18="",F18=""),"",IF(I18="Annuler","✗ À annuler sous "&amp;(IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G18=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H18&lt;&gt;"",TODAY()-H18&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H18)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B18="",F18=""),"",IF(I18="Annuler","À annuler sous "&amp;(IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G18="Oui","Fin de l'essai dans "&amp;(IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H18&lt;&gt;"",TODAY()-H18&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H18)&amp;" jours","Renouvellement dans "&amp;(IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F18&gt;=TODAY(),F18,IF(E18="Hebdo",F18+7*ROUNDUP((TODAY()-F18)/7,0),EDATE(F18,IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12))*ROUNDUP((DATEDIF(F18,TODAY(),"m")+1)/IF(E18="Mensuel",1,IF(E18="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M18" s="1" t="n"/>
@@ -2480,7 +2516,7 @@
         <v/>
       </c>
       <c r="L19" s="26">
-        <f>IF(OR(B19="",F19=""),"",IF(I19="Annuler","✗ À annuler sous "&amp;(IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G19=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H19&lt;&gt;"",TODAY()-H19&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H19)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B19="",F19=""),"",IF(I19="Annuler","À annuler sous "&amp;(IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G19="Oui","Fin de l'essai dans "&amp;(IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H19&lt;&gt;"",TODAY()-H19&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H19)&amp;" jours","Renouvellement dans "&amp;(IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F19&gt;=TODAY(),F19,IF(E19="Hebdo",F19+7*ROUNDUP((TODAY()-F19)/7,0),EDATE(F19,IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12))*ROUNDUP((DATEDIF(F19,TODAY(),"m")+1)/IF(E19="Mensuel",1,IF(E19="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M19" s="1" t="n"/>
@@ -2504,7 +2540,7 @@
         <v/>
       </c>
       <c r="L20" s="26">
-        <f>IF(OR(B20="",F20=""),"",IF(I20="Annuler","✗ À annuler sous "&amp;(IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G20=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H20&lt;&gt;"",TODAY()-H20&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H20)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B20="",F20=""),"",IF(I20="Annuler","À annuler sous "&amp;(IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G20="Oui","Fin de l'essai dans "&amp;(IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H20&lt;&gt;"",TODAY()-H20&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H20)&amp;" jours","Renouvellement dans "&amp;(IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F20&gt;=TODAY(),F20,IF(E20="Hebdo",F20+7*ROUNDUP((TODAY()-F20)/7,0),EDATE(F20,IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12))*ROUNDUP((DATEDIF(F20,TODAY(),"m")+1)/IF(E20="Mensuel",1,IF(E20="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M20" s="1" t="n"/>
@@ -2528,7 +2564,7 @@
         <v/>
       </c>
       <c r="L21" s="26">
-        <f>IF(OR(B21="",F21=""),"",IF(I21="Annuler","✗ À annuler sous "&amp;(IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G21=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H21&lt;&gt;"",TODAY()-H21&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H21)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B21="",F21=""),"",IF(I21="Annuler","À annuler sous "&amp;(IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G21="Oui","Fin de l'essai dans "&amp;(IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H21&lt;&gt;"",TODAY()-H21&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H21)&amp;" jours","Renouvellement dans "&amp;(IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F21&gt;=TODAY(),F21,IF(E21="Hebdo",F21+7*ROUNDUP((TODAY()-F21)/7,0),EDATE(F21,IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12))*ROUNDUP((DATEDIF(F21,TODAY(),"m")+1)/IF(E21="Mensuel",1,IF(E21="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M21" s="1" t="n"/>
@@ -2552,7 +2588,7 @@
         <v/>
       </c>
       <c r="L22" s="26">
-        <f>IF(OR(B22="",F22=""),"",IF(I22="Annuler","✗ À annuler sous "&amp;(IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G22=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H22&lt;&gt;"",TODAY()-H22&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H22)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B22="",F22=""),"",IF(I22="Annuler","À annuler sous "&amp;(IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G22="Oui","Fin de l'essai dans "&amp;(IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H22&lt;&gt;"",TODAY()-H22&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H22)&amp;" jours","Renouvellement dans "&amp;(IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F22&gt;=TODAY(),F22,IF(E22="Hebdo",F22+7*ROUNDUP((TODAY()-F22)/7,0),EDATE(F22,IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12))*ROUNDUP((DATEDIF(F22,TODAY(),"m")+1)/IF(E22="Mensuel",1,IF(E22="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M22" s="1" t="n"/>
@@ -2576,7 +2612,7 @@
         <v/>
       </c>
       <c r="L23" s="26">
-        <f>IF(OR(B23="",F23=""),"",IF(I23="Annuler","✗ À annuler sous "&amp;(IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G23=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H23&lt;&gt;"",TODAY()-H23&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H23)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B23="",F23=""),"",IF(I23="Annuler","À annuler sous "&amp;(IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G23="Oui","Fin de l'essai dans "&amp;(IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H23&lt;&gt;"",TODAY()-H23&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H23)&amp;" jours","Renouvellement dans "&amp;(IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F23&gt;=TODAY(),F23,IF(E23="Hebdo",F23+7*ROUNDUP((TODAY()-F23)/7,0),EDATE(F23,IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12))*ROUNDUP((DATEDIF(F23,TODAY(),"m")+1)/IF(E23="Mensuel",1,IF(E23="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M23" s="1" t="n"/>
@@ -2600,7 +2636,7 @@
         <v/>
       </c>
       <c r="L24" s="26">
-        <f>IF(OR(B24="",F24=""),"",IF(I24="Annuler","✗ À annuler sous "&amp;(IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G24=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H24&lt;&gt;"",TODAY()-H24&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H24)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B24="",F24=""),"",IF(I24="Annuler","À annuler sous "&amp;(IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G24="Oui","Fin de l'essai dans "&amp;(IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H24&lt;&gt;"",TODAY()-H24&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H24)&amp;" jours","Renouvellement dans "&amp;(IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F24&gt;=TODAY(),F24,IF(E24="Hebdo",F24+7*ROUNDUP((TODAY()-F24)/7,0),EDATE(F24,IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12))*ROUNDUP((DATEDIF(F24,TODAY(),"m")+1)/IF(E24="Mensuel",1,IF(E24="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M24" s="1" t="n"/>
@@ -2624,7 +2660,7 @@
         <v/>
       </c>
       <c r="L25" s="26">
-        <f>IF(OR(B25="",F25=""),"",IF(I25="Annuler","✗ À annuler sous "&amp;(IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G25=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H25&lt;&gt;"",TODAY()-H25&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H25)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B25="",F25=""),"",IF(I25="Annuler","À annuler sous "&amp;(IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G25="Oui","Fin de l'essai dans "&amp;(IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H25&lt;&gt;"",TODAY()-H25&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H25)&amp;" jours","Renouvellement dans "&amp;(IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F25&gt;=TODAY(),F25,IF(E25="Hebdo",F25+7*ROUNDUP((TODAY()-F25)/7,0),EDATE(F25,IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12))*ROUNDUP((DATEDIF(F25,TODAY(),"m")+1)/IF(E25="Mensuel",1,IF(E25="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M25" s="1" t="n"/>
@@ -2648,7 +2684,7 @@
         <v/>
       </c>
       <c r="L26" s="26">
-        <f>IF(OR(B26="",F26=""),"",IF(I26="Annuler","✗ À annuler sous "&amp;(IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G26=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H26&lt;&gt;"",TODAY()-H26&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H26)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B26="",F26=""),"",IF(I26="Annuler","À annuler sous "&amp;(IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G26="Oui","Fin de l'essai dans "&amp;(IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H26&lt;&gt;"",TODAY()-H26&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H26)&amp;" jours","Renouvellement dans "&amp;(IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F26&gt;=TODAY(),F26,IF(E26="Hebdo",F26+7*ROUNDUP((TODAY()-F26)/7,0),EDATE(F26,IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12))*ROUNDUP((DATEDIF(F26,TODAY(),"m")+1)/IF(E26="Mensuel",1,IF(E26="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M26" s="1" t="n"/>
@@ -2672,7 +2708,7 @@
         <v/>
       </c>
       <c r="L27" s="26">
-        <f>IF(OR(B27="",F27=""),"",IF(I27="Annuler","✗ À annuler sous "&amp;(IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G27=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H27&lt;&gt;"",TODAY()-H27&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H27)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B27="",F27=""),"",IF(I27="Annuler","À annuler sous "&amp;(IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G27="Oui","Fin de l'essai dans "&amp;(IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H27&lt;&gt;"",TODAY()-H27&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H27)&amp;" jours","Renouvellement dans "&amp;(IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F27&gt;=TODAY(),F27,IF(E27="Hebdo",F27+7*ROUNDUP((TODAY()-F27)/7,0),EDATE(F27,IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12))*ROUNDUP((DATEDIF(F27,TODAY(),"m")+1)/IF(E27="Mensuel",1,IF(E27="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M27" s="1" t="n"/>
@@ -2696,7 +2732,7 @@
         <v/>
       </c>
       <c r="L28" s="26">
-        <f>IF(OR(B28="",F28=""),"",IF(I28="Annuler","✗ À annuler sous "&amp;(IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G28=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H28&lt;&gt;"",TODAY()-H28&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H28)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B28="",F28=""),"",IF(I28="Annuler","À annuler sous "&amp;(IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G28="Oui","Fin de l'essai dans "&amp;(IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H28&lt;&gt;"",TODAY()-H28&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H28)&amp;" jours","Renouvellement dans "&amp;(IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F28&gt;=TODAY(),F28,IF(E28="Hebdo",F28+7*ROUNDUP((TODAY()-F28)/7,0),EDATE(F28,IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12))*ROUNDUP((DATEDIF(F28,TODAY(),"m")+1)/IF(E28="Mensuel",1,IF(E28="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M28" s="1" t="n"/>
@@ -2720,7 +2756,7 @@
         <v/>
       </c>
       <c r="L29" s="26">
-        <f>IF(OR(B29="",F29=""),"",IF(I29="Annuler","✗ À annuler sous "&amp;(IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G29=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H29&lt;&gt;"",TODAY()-H29&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H29)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B29="",F29=""),"",IF(I29="Annuler","À annuler sous "&amp;(IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G29="Oui","Fin de l'essai dans "&amp;(IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H29&lt;&gt;"",TODAY()-H29&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H29)&amp;" jours","Renouvellement dans "&amp;(IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F29&gt;=TODAY(),F29,IF(E29="Hebdo",F29+7*ROUNDUP((TODAY()-F29)/7,0),EDATE(F29,IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12))*ROUNDUP((DATEDIF(F29,TODAY(),"m")+1)/IF(E29="Mensuel",1,IF(E29="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M29" s="1" t="n"/>
@@ -2744,7 +2780,7 @@
         <v/>
       </c>
       <c r="L30" s="26">
-        <f>IF(OR(B30="",F30=""),"",IF(I30="Annuler","✗ À annuler sous "&amp;(IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G30=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H30&lt;&gt;"",TODAY()-H30&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H30)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B30="",F30=""),"",IF(I30="Annuler","À annuler sous "&amp;(IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G30="Oui","Fin de l'essai dans "&amp;(IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H30&lt;&gt;"",TODAY()-H30&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H30)&amp;" jours","Renouvellement dans "&amp;(IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F30&gt;=TODAY(),F30,IF(E30="Hebdo",F30+7*ROUNDUP((TODAY()-F30)/7,0),EDATE(F30,IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12))*ROUNDUP((DATEDIF(F30,TODAY(),"m")+1)/IF(E30="Mensuel",1,IF(E30="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M30" s="1" t="n"/>
@@ -2768,7 +2804,7 @@
         <v/>
       </c>
       <c r="L31" s="26">
-        <f>IF(OR(B31="",F31=""),"",IF(I31="Annuler","✗ À annuler sous "&amp;(IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G31=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H31&lt;&gt;"",TODAY()-H31&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H31)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B31="",F31=""),"",IF(I31="Annuler","À annuler sous "&amp;(IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G31="Oui","Fin de l'essai dans "&amp;(IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H31&lt;&gt;"",TODAY()-H31&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H31)&amp;" jours","Renouvellement dans "&amp;(IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F31&gt;=TODAY(),F31,IF(E31="Hebdo",F31+7*ROUNDUP((TODAY()-F31)/7,0),EDATE(F31,IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12))*ROUNDUP((DATEDIF(F31,TODAY(),"m")+1)/IF(E31="Mensuel",1,IF(E31="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M31" s="1" t="n"/>
@@ -2792,7 +2828,7 @@
         <v/>
       </c>
       <c r="L32" s="26">
-        <f>IF(OR(B32="",F32=""),"",IF(I32="Annuler","✗ À annuler sous "&amp;(IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G32=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H32&lt;&gt;"",TODAY()-H32&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H32)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B32="",F32=""),"",IF(I32="Annuler","À annuler sous "&amp;(IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G32="Oui","Fin de l'essai dans "&amp;(IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H32&lt;&gt;"",TODAY()-H32&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H32)&amp;" jours","Renouvellement dans "&amp;(IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F32&gt;=TODAY(),F32,IF(E32="Hebdo",F32+7*ROUNDUP((TODAY()-F32)/7,0),EDATE(F32,IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12))*ROUNDUP((DATEDIF(F32,TODAY(),"m")+1)/IF(E32="Mensuel",1,IF(E32="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M32" s="1" t="n"/>
@@ -2816,7 +2852,7 @@
         <v/>
       </c>
       <c r="L33" s="26">
-        <f>IF(OR(B33="",F33=""),"",IF(I33="Annuler","✗ À annuler sous "&amp;(IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G33=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H33&lt;&gt;"",TODAY()-H33&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H33)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B33="",F33=""),"",IF(I33="Annuler","À annuler sous "&amp;(IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G33="Oui","Fin de l'essai dans "&amp;(IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H33&lt;&gt;"",TODAY()-H33&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H33)&amp;" jours","Renouvellement dans "&amp;(IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F33&gt;=TODAY(),F33,IF(E33="Hebdo",F33+7*ROUNDUP((TODAY()-F33)/7,0),EDATE(F33,IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12))*ROUNDUP((DATEDIF(F33,TODAY(),"m")+1)/IF(E33="Mensuel",1,IF(E33="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M33" s="1" t="n"/>
@@ -2840,7 +2876,7 @@
         <v/>
       </c>
       <c r="L34" s="26">
-        <f>IF(OR(B34="",F34=""),"",IF(I34="Annuler","✗ À annuler sous "&amp;(IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G34=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H34&lt;&gt;"",TODAY()-H34&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H34)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B34="",F34=""),"",IF(I34="Annuler","À annuler sous "&amp;(IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G34="Oui","Fin de l'essai dans "&amp;(IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H34&lt;&gt;"",TODAY()-H34&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H34)&amp;" jours","Renouvellement dans "&amp;(IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F34&gt;=TODAY(),F34,IF(E34="Hebdo",F34+7*ROUNDUP((TODAY()-F34)/7,0),EDATE(F34,IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12))*ROUNDUP((DATEDIF(F34,TODAY(),"m")+1)/IF(E34="Mensuel",1,IF(E34="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M34" s="1" t="n"/>
@@ -2864,7 +2900,7 @@
         <v/>
       </c>
       <c r="L35" s="26">
-        <f>IF(OR(B35="",F35=""),"",IF(I35="Annuler","✗ À annuler sous "&amp;(IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G35=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H35&lt;&gt;"",TODAY()-H35&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H35)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B35="",F35=""),"",IF(I35="Annuler","À annuler sous "&amp;(IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G35="Oui","Fin de l'essai dans "&amp;(IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H35&lt;&gt;"",TODAY()-H35&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H35)&amp;" jours","Renouvellement dans "&amp;(IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F35&gt;=TODAY(),F35,IF(E35="Hebdo",F35+7*ROUNDUP((TODAY()-F35)/7,0),EDATE(F35,IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12))*ROUNDUP((DATEDIF(F35,TODAY(),"m")+1)/IF(E35="Mensuel",1,IF(E35="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M35" s="1" t="n"/>
@@ -2888,7 +2924,7 @@
         <v/>
       </c>
       <c r="L36" s="26">
-        <f>IF(OR(B36="",F36=""),"",IF(I36="Annuler","✗ À annuler sous "&amp;(IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G36=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H36&lt;&gt;"",TODAY()-H36&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H36)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B36="",F36=""),"",IF(I36="Annuler","À annuler sous "&amp;(IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G36="Oui","Fin de l'essai dans "&amp;(IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H36&lt;&gt;"",TODAY()-H36&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H36)&amp;" jours","Renouvellement dans "&amp;(IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F36&gt;=TODAY(),F36,IF(E36="Hebdo",F36+7*ROUNDUP((TODAY()-F36)/7,0),EDATE(F36,IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12))*ROUNDUP((DATEDIF(F36,TODAY(),"m")+1)/IF(E36="Mensuel",1,IF(E36="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M36" s="1" t="n"/>
@@ -2912,7 +2948,7 @@
         <v/>
       </c>
       <c r="L37" s="26">
-        <f>IF(OR(B37="",F37=""),"",IF(I37="Annuler","✗ À annuler sous "&amp;(IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G37=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H37&lt;&gt;"",TODAY()-H37&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H37)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B37="",F37=""),"",IF(I37="Annuler","À annuler sous "&amp;(IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G37="Oui","Fin de l'essai dans "&amp;(IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H37&lt;&gt;"",TODAY()-H37&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H37)&amp;" jours","Renouvellement dans "&amp;(IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F37&gt;=TODAY(),F37,IF(E37="Hebdo",F37+7*ROUNDUP((TODAY()-F37)/7,0),EDATE(F37,IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12))*ROUNDUP((DATEDIF(F37,TODAY(),"m")+1)/IF(E37="Mensuel",1,IF(E37="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M37" s="1" t="n"/>
@@ -2936,7 +2972,7 @@
         <v/>
       </c>
       <c r="L38" s="26">
-        <f>IF(OR(B38="",F38=""),"",IF(I38="Annuler","✗ À annuler sous "&amp;(IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G38=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H38&lt;&gt;"",TODAY()-H38&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H38)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B38="",F38=""),"",IF(I38="Annuler","À annuler sous "&amp;(IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G38="Oui","Fin de l'essai dans "&amp;(IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H38&lt;&gt;"",TODAY()-H38&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H38)&amp;" jours","Renouvellement dans "&amp;(IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F38&gt;=TODAY(),F38,IF(E38="Hebdo",F38+7*ROUNDUP((TODAY()-F38)/7,0),EDATE(F38,IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12))*ROUNDUP((DATEDIF(F38,TODAY(),"m")+1)/IF(E38="Mensuel",1,IF(E38="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M38" s="1" t="n"/>
@@ -2960,7 +2996,7 @@
         <v/>
       </c>
       <c r="L39" s="26">
-        <f>IF(OR(B39="",F39=""),"",IF(I39="Annuler","✗ À annuler sous "&amp;(IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G39=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H39&lt;&gt;"",TODAY()-H39&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H39)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B39="",F39=""),"",IF(I39="Annuler","À annuler sous "&amp;(IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G39="Oui","Fin de l'essai dans "&amp;(IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H39&lt;&gt;"",TODAY()-H39&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H39)&amp;" jours","Renouvellement dans "&amp;(IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F39&gt;=TODAY(),F39,IF(E39="Hebdo",F39+7*ROUNDUP((TODAY()-F39)/7,0),EDATE(F39,IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12))*ROUNDUP((DATEDIF(F39,TODAY(),"m")+1)/IF(E39="Mensuel",1,IF(E39="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M39" s="1" t="n"/>
@@ -2984,7 +3020,7 @@
         <v/>
       </c>
       <c r="L40" s="26">
-        <f>IF(OR(B40="",F40=""),"",IF(I40="Annuler","✗ À annuler sous "&amp;(IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G40=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H40&lt;&gt;"",TODAY()-H40&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H40)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B40="",F40=""),"",IF(I40="Annuler","À annuler sous "&amp;(IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G40="Oui","Fin de l'essai dans "&amp;(IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H40&lt;&gt;"",TODAY()-H40&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H40)&amp;" jours","Renouvellement dans "&amp;(IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F40&gt;=TODAY(),F40,IF(E40="Hebdo",F40+7*ROUNDUP((TODAY()-F40)/7,0),EDATE(F40,IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12))*ROUNDUP((DATEDIF(F40,TODAY(),"m")+1)/IF(E40="Mensuel",1,IF(E40="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M40" s="1" t="n"/>
@@ -3008,7 +3044,7 @@
         <v/>
       </c>
       <c r="L41" s="26">
-        <f>IF(OR(B41="",F41=""),"",IF(I41="Annuler","✗ À annuler sous "&amp;(IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G41=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H41&lt;&gt;"",TODAY()-H41&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H41)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B41="",F41=""),"",IF(I41="Annuler","À annuler sous "&amp;(IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G41="Oui","Fin de l'essai dans "&amp;(IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H41&lt;&gt;"",TODAY()-H41&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H41)&amp;" jours","Renouvellement dans "&amp;(IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F41&gt;=TODAY(),F41,IF(E41="Hebdo",F41+7*ROUNDUP((TODAY()-F41)/7,0),EDATE(F41,IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12))*ROUNDUP((DATEDIF(F41,TODAY(),"m")+1)/IF(E41="Mensuel",1,IF(E41="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M41" s="1" t="n"/>
@@ -3032,7 +3068,7 @@
         <v/>
       </c>
       <c r="L42" s="26">
-        <f>IF(OR(B42="",F42=""),"",IF(I42="Annuler","✗ À annuler sous "&amp;(IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G42=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H42&lt;&gt;"",TODAY()-H42&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H42)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B42="",F42=""),"",IF(I42="Annuler","À annuler sous "&amp;(IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G42="Oui","Fin de l'essai dans "&amp;(IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H42&lt;&gt;"",TODAY()-H42&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H42)&amp;" jours","Renouvellement dans "&amp;(IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F42&gt;=TODAY(),F42,IF(E42="Hebdo",F42+7*ROUNDUP((TODAY()-F42)/7,0),EDATE(F42,IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12))*ROUNDUP((DATEDIF(F42,TODAY(),"m")+1)/IF(E42="Mensuel",1,IF(E42="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M42" s="1" t="n"/>
@@ -3056,7 +3092,7 @@
         <v/>
       </c>
       <c r="L43" s="26">
-        <f>IF(OR(B43="",F43=""),"",IF(I43="Annuler","✗ À annuler sous "&amp;(IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G43=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H43&lt;&gt;"",TODAY()-H43&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H43)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B43="",F43=""),"",IF(I43="Annuler","À annuler sous "&amp;(IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G43="Oui","Fin de l'essai dans "&amp;(IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H43&lt;&gt;"",TODAY()-H43&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H43)&amp;" jours","Renouvellement dans "&amp;(IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F43&gt;=TODAY(),F43,IF(E43="Hebdo",F43+7*ROUNDUP((TODAY()-F43)/7,0),EDATE(F43,IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12))*ROUNDUP((DATEDIF(F43,TODAY(),"m")+1)/IF(E43="Mensuel",1,IF(E43="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M43" s="1" t="n"/>
@@ -3080,7 +3116,7 @@
         <v/>
       </c>
       <c r="L44" s="26">
-        <f>IF(OR(B44="",F44=""),"",IF(I44="Annuler","✗ À annuler sous "&amp;(IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G44=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H44&lt;&gt;"",TODAY()-H44&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H44)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B44="",F44=""),"",IF(I44="Annuler","À annuler sous "&amp;(IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G44="Oui","Fin de l'essai dans "&amp;(IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H44&lt;&gt;"",TODAY()-H44&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H44)&amp;" jours","Renouvellement dans "&amp;(IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F44&gt;=TODAY(),F44,IF(E44="Hebdo",F44+7*ROUNDUP((TODAY()-F44)/7,0),EDATE(F44,IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12))*ROUNDUP((DATEDIF(F44,TODAY(),"m")+1)/IF(E44="Mensuel",1,IF(E44="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M44" s="1" t="n"/>
@@ -3104,7 +3140,7 @@
         <v/>
       </c>
       <c r="L45" s="26">
-        <f>IF(OR(B45="",F45=""),"",IF(I45="Annuler","✗ À annuler sous "&amp;(IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G45=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H45&lt;&gt;"",TODAY()-H45&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H45)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B45="",F45=""),"",IF(I45="Annuler","À annuler sous "&amp;(IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G45="Oui","Fin de l'essai dans "&amp;(IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H45&lt;&gt;"",TODAY()-H45&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H45)&amp;" jours","Renouvellement dans "&amp;(IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F45&gt;=TODAY(),F45,IF(E45="Hebdo",F45+7*ROUNDUP((TODAY()-F45)/7,0),EDATE(F45,IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12))*ROUNDUP((DATEDIF(F45,TODAY(),"m")+1)/IF(E45="Mensuel",1,IF(E45="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M45" s="1" t="n"/>
@@ -3128,7 +3164,7 @@
         <v/>
       </c>
       <c r="L46" s="26">
-        <f>IF(OR(B46="",F46=""),"",IF(I46="Annuler","✗ À annuler sous "&amp;(IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G46=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H46&lt;&gt;"",TODAY()-H46&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H46)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B46="",F46=""),"",IF(I46="Annuler","À annuler sous "&amp;(IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G46="Oui","Fin de l'essai dans "&amp;(IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H46&lt;&gt;"",TODAY()-H46&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H46)&amp;" jours","Renouvellement dans "&amp;(IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F46&gt;=TODAY(),F46,IF(E46="Hebdo",F46+7*ROUNDUP((TODAY()-F46)/7,0),EDATE(F46,IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12))*ROUNDUP((DATEDIF(F46,TODAY(),"m")+1)/IF(E46="Mensuel",1,IF(E46="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M46" s="1" t="n"/>
@@ -3152,7 +3188,7 @@
         <v/>
       </c>
       <c r="L47" s="26">
-        <f>IF(OR(B47="",F47=""),"",IF(I47="Annuler","✗ À annuler sous "&amp;(IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G47=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H47&lt;&gt;"",TODAY()-H47&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H47)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B47="",F47=""),"",IF(I47="Annuler","À annuler sous "&amp;(IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G47="Oui","Fin de l'essai dans "&amp;(IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H47&lt;&gt;"",TODAY()-H47&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H47)&amp;" jours","Renouvellement dans "&amp;(IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F47&gt;=TODAY(),F47,IF(E47="Hebdo",F47+7*ROUNDUP((TODAY()-F47)/7,0),EDATE(F47,IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12))*ROUNDUP((DATEDIF(F47,TODAY(),"m")+1)/IF(E47="Mensuel",1,IF(E47="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M47" s="1" t="n"/>
@@ -3176,7 +3212,7 @@
         <v/>
       </c>
       <c r="L48" s="26">
-        <f>IF(OR(B48="",F48=""),"",IF(I48="Annuler","✗ À annuler sous "&amp;(IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G48=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H48&lt;&gt;"",TODAY()-H48&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H48)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B48="",F48=""),"",IF(I48="Annuler","À annuler sous "&amp;(IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G48="Oui","Fin de l'essai dans "&amp;(IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H48&lt;&gt;"",TODAY()-H48&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H48)&amp;" jours","Renouvellement dans "&amp;(IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F48&gt;=TODAY(),F48,IF(E48="Hebdo",F48+7*ROUNDUP((TODAY()-F48)/7,0),EDATE(F48,IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12))*ROUNDUP((DATEDIF(F48,TODAY(),"m")+1)/IF(E48="Mensuel",1,IF(E48="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M48" s="1" t="n"/>
@@ -3200,7 +3236,7 @@
         <v/>
       </c>
       <c r="L49" s="26">
-        <f>IF(OR(B49="",F49=""),"",IF(I49="Annuler","✗ À annuler sous "&amp;(IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G49=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H49&lt;&gt;"",TODAY()-H49&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H49)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B49="",F49=""),"",IF(I49="Annuler","À annuler sous "&amp;(IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G49="Oui","Fin de l'essai dans "&amp;(IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H49&lt;&gt;"",TODAY()-H49&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H49)&amp;" jours","Renouvellement dans "&amp;(IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F49&gt;=TODAY(),F49,IF(E49="Hebdo",F49+7*ROUNDUP((TODAY()-F49)/7,0),EDATE(F49,IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12))*ROUNDUP((DATEDIF(F49,TODAY(),"m")+1)/IF(E49="Mensuel",1,IF(E49="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M49" s="1" t="n"/>
@@ -3224,7 +3260,7 @@
         <v/>
       </c>
       <c r="L50" s="26">
-        <f>IF(OR(B50="",F50=""),"",IF(I50="Annuler","✗ À annuler sous "&amp;(IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G50=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H50&lt;&gt;"",TODAY()-H50&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H50)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B50="",F50=""),"",IF(I50="Annuler","À annuler sous "&amp;(IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G50="Oui","Fin de l'essai dans "&amp;(IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H50&lt;&gt;"",TODAY()-H50&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H50)&amp;" jours","Renouvellement dans "&amp;(IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F50&gt;=TODAY(),F50,IF(E50="Hebdo",F50+7*ROUNDUP((TODAY()-F50)/7,0),EDATE(F50,IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12))*ROUNDUP((DATEDIF(F50,TODAY(),"m")+1)/IF(E50="Mensuel",1,IF(E50="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M50" s="1" t="n"/>
@@ -3248,7 +3284,7 @@
         <v/>
       </c>
       <c r="L51" s="26">
-        <f>IF(OR(B51="",F51=""),"",IF(I51="Annuler","✗ À annuler sous "&amp;(IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G51=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H51&lt;&gt;"",TODAY()-H51&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H51)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B51="",F51=""),"",IF(I51="Annuler","À annuler sous "&amp;(IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G51="Oui","Fin de l'essai dans "&amp;(IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H51&lt;&gt;"",TODAY()-H51&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H51)&amp;" jours","Renouvellement dans "&amp;(IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F51&gt;=TODAY(),F51,IF(E51="Hebdo",F51+7*ROUNDUP((TODAY()-F51)/7,0),EDATE(F51,IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12))*ROUNDUP((DATEDIF(F51,TODAY(),"m")+1)/IF(E51="Mensuel",1,IF(E51="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M51" s="1" t="n"/>
@@ -3272,7 +3308,7 @@
         <v/>
       </c>
       <c r="L52" s="26">
-        <f>IF(OR(B52="",F52=""),"",IF(I52="Annuler","✗ À annuler sous "&amp;(IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G52=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H52&lt;&gt;"",TODAY()-H52&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H52)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B52="",F52=""),"",IF(I52="Annuler","À annuler sous "&amp;(IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G52="Oui","Fin de l'essai dans "&amp;(IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H52&lt;&gt;"",TODAY()-H52&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H52)&amp;" jours","Renouvellement dans "&amp;(IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F52&gt;=TODAY(),F52,IF(E52="Hebdo",F52+7*ROUNDUP((TODAY()-F52)/7,0),EDATE(F52,IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12))*ROUNDUP((DATEDIF(F52,TODAY(),"m")+1)/IF(E52="Mensuel",1,IF(E52="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M52" s="1" t="n"/>
@@ -3296,7 +3332,7 @@
         <v/>
       </c>
       <c r="L53" s="26">
-        <f>IF(OR(B53="",F53=""),"",IF(I53="Annuler","✗ À annuler sous "&amp;(IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G53=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H53&lt;&gt;"",TODAY()-H53&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H53)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B53="",F53=""),"",IF(I53="Annuler","À annuler sous "&amp;(IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G53="Oui","Fin de l'essai dans "&amp;(IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H53&lt;&gt;"",TODAY()-H53&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H53)&amp;" jours","Renouvellement dans "&amp;(IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F53&gt;=TODAY(),F53,IF(E53="Hebdo",F53+7*ROUNDUP((TODAY()-F53)/7,0),EDATE(F53,IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12))*ROUNDUP((DATEDIF(F53,TODAY(),"m")+1)/IF(E53="Mensuel",1,IF(E53="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M53" s="1" t="n"/>
@@ -3320,7 +3356,7 @@
         <v/>
       </c>
       <c r="L54" s="26">
-        <f>IF(OR(B54="",F54=""),"",IF(I54="Annuler","✗ À annuler sous "&amp;(IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G54=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H54&lt;&gt;"",TODAY()-H54&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H54)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B54="",F54=""),"",IF(I54="Annuler","À annuler sous "&amp;(IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G54="Oui","Fin de l'essai dans "&amp;(IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H54&lt;&gt;"",TODAY()-H54&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H54)&amp;" jours","Renouvellement dans "&amp;(IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F54&gt;=TODAY(),F54,IF(E54="Hebdo",F54+7*ROUNDUP((TODAY()-F54)/7,0),EDATE(F54,IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12))*ROUNDUP((DATEDIF(F54,TODAY(),"m")+1)/IF(E54="Mensuel",1,IF(E54="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M54" s="1" t="n"/>
@@ -3344,7 +3380,7 @@
         <v/>
       </c>
       <c r="L55" s="26">
-        <f>IF(OR(B55="",F55=""),"",IF(I55="Annuler","✗ À annuler sous "&amp;(IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(G55=TRUE,"⚠ Fin de l’essai dans "&amp;(IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)",IF(AND(H55&lt;&gt;"",TODAY()-H55&gt;30),"💤 Pas utilisé depuis "&amp;(TODAY()-H55)&amp;" jours : ça vaut encore le coup ?","Renouvellement dans "&amp;(IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&amp;" jour(s)"))))</f>
+        <f>IF(OR(B55="",F55=""),"",IF(I55="Annuler","À annuler sous "&amp;(IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(G55="Oui","Fin de l'essai dans "&amp;(IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours"),IF(AND(H55&lt;&gt;"",TODAY()-H55&gt;30),"Pas utilisé depuis "&amp;(TODAY()-H55)&amp;" jours","Renouvellement dans "&amp;(IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&amp;IF((IF(F55&gt;=TODAY(),F55,IF(E55="Hebdo",F55+7*ROUNDUP((TODAY()-F55)/7,0),EDATE(F55,IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12))*ROUNDUP((DATEDIF(F55,TODAY(),"m")+1)/IF(E55="Mensuel",1,IF(E55="Trimestriel",3,12)),0))))-TODAY())&lt;=1," jour"," jours")))))</f>
         <v/>
       </c>
       <c r="M55" s="1" t="n"/>
@@ -3711,16 +3747,16 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="L6:L55">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>LEFT($L6,1)="✗"</formula>
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>LEFT($L6,9)="À annuler"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>LEFT($L6,1)="⚠"</formula>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>LEFT($L6,6)="Fin de"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
-      <formula>LEFT($L6,2)="💤"</formula>
+    <cfRule type="expression" priority="3" dxfId="3">
+      <formula>LEFT($L6,3)="Pas"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3">
+    <cfRule type="expression" priority="4" dxfId="0">
       <formula>LEFT($L6,6)="Renouv"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3732,7 +3768,7 @@
       <formula1>"Hebdo,Mensuel,Trimestriel,Annuel"</formula1>
     </dataValidation>
     <dataValidation sqref="G6:G55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
+      <formula1>"Oui,Non"</formula1>
     </dataValidation>
     <dataValidation sqref="I6:I55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Garder,Annuler,Décider"</formula1>
@@ -3767,7 +3803,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Commencer ici : 2 minutes</t>
+          <t>Commencer ici</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -3777,7 +3813,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Tapez uniquement dans les cases JAUNES.</t>
+          <t>Tapez uniquement dans les cases jaunes. Tout le reste est calculé.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -3798,7 +3834,7 @@
       </c>
       <c r="C5" s="28" t="inlineStr">
         <is>
-          <t>Onglet Abonnements : ajoutez chaque abonnement (relevé bancaire + magasin d’applis du téléphone pour les retrouver).</t>
+          <t>Onglet Abonnements : ajoutez chaque abonnement. Le relevé bancaire et le magasin d'applis du téléphone aident à les retrouver.</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
@@ -3838,7 +3874,7 @@
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>Essai gratuit ? Mettez TRUE : alerte rouge avec les jours restants avant le premier débit.</t>
+          <t>Essai gratuit : choisissez Oui et le statut passe en rouge, avec les jours restants avant le premier débit.</t>
         </is>
       </c>
       <c r="D9" s="1" t="n"/>
@@ -3858,7 +3894,7 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>Dernière utilisation : mettez-la à jour de temps en temps. Plus de 30 jours = orange.</t>
+          <t>Dernière utilisation : mettez-la à jour de temps en temps. Après 30 jours sans utilisation, le statut passe en orange.</t>
         </is>
       </c>
       <c r="D11" s="1" t="n"/>
@@ -3878,7 +3914,7 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>Garder ? Choisissez Garder, Annuler ou Décider. Le Tableau de bord montre l’économie par an.</t>
+          <t>Garder : choisissez Garder, Annuler ou Décider. Le Tableau de bord montre l'économie par an.</t>
         </is>
       </c>
       <c r="D13" s="1" t="n"/>
@@ -3906,7 +3942,7 @@
       <c r="B17" s="1" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Les lignes d’exemple montrent comment ça marche. Supprimez-les et ajoutez les vôtres.</t>
+          <t>Les lignes d'exemple montrent comment ça marche. Supprimez-les et ajoutez les vôtres.</t>
         </is>
       </c>
       <c r="D17" s="1" t="n"/>
@@ -3922,7 +3958,7 @@
       <c r="B19" s="1" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Fonctionne dans Google Sheets (importez dans Drive, puis Fichier → Enregistrer au format Google Sheets) et dans Microsoft Excel.</t>
+          <t>Fonctionne dans Google Sheets (importez-le dans Drive, puis Fichier &gt; Enregistrer au format Google Sheets) et dans Microsoft Excel.</t>
         </is>
       </c>
       <c r="D19" s="1" t="n"/>

</xml_diff>